<commit_message>
feat(deal-mgmt/marketing): GP 로고 URL 수집 스크립트 및 데이터 추가
- fetch_gp_logos.py: Clearbit/og:image/DuckDuckGo 3단계 폴백으로 GP 로고 URL 자동 수집
- MA_GP_v3.xlsx: O열에 GP CI 로고 URL 입력 (seed_gp_profiles.py --force로 DB 반영 필요)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deal-mgmt/data/MA_GP_v3.xlsx
+++ b/deal-mgmt/data/MA_GP_v3.xlsx
@@ -1385,6 +1385,11 @@
           <t>전력기자재, 조선/해양, 물류/터미널, 구조조정 | 투자기업: 우진기전, 성동조선해양, 성운탱크터미널</t>
         </is>
       </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>http://curiouspe.com/images/logo_b.png</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="6" t="n">
@@ -1433,6 +1438,11 @@
           <t>IT, 2차전지, 반도체, 그로스에쿼티 | 투자기업: 미래첨단소재</t>
         </is>
       </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>http://www.dominusinvestment.com/public/images/cm_logo_1.png</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="25.5" customHeight="1">
       <c r="A23" s="6" t="n">
@@ -1481,6 +1491,11 @@
           <t>골프/스포츠, 레저, 첨단소재 | 투자기업: 테일러메이드, 사우스스프링스CC, 코오롱첨단소재</t>
         </is>
       </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>https://framerusercontent.com/images/jObioPBZxAWixH7mYiMVRJYFKpg.png</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="25.5" customHeight="1">
       <c r="A24" s="6" t="n">
@@ -1529,6 +1544,11 @@
           <t>반도체장비, 전자부품/제조, IT보안 | 투자기업: 한미반도체, 서진시스템, 윈스, 모델솔루션</t>
         </is>
       </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>https://crescendoep.com/wp-content/uploads/2023/06/logo-6.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="25.5" customHeight="1">
       <c r="A25" s="6" t="n">
@@ -2259,6 +2279,11 @@
           <t>모빌리티, 금융/보험, 항공, 바이아웃 | 투자기업: 카카오모빌리티, MG손해보험, 에어프리마, 황조</t>
         </is>
       </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>https://www.jcpartners.kr/wp-content/uploads/2020/12/web-agency-logo-3.png</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="6" t="n">
@@ -2355,6 +2380,11 @@
           <t>플랫폼, 콘텐츠, 보안, 제조, 냉동식품 | 투자기업: 원스토어, 콘텐츠웨이브, ADT캡스, 제일기공, 강동냉장</t>
         </is>
       </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>http://www.skspe.com/bc.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="25.5" customHeight="1">
       <c r="A42" s="6" t="n">
@@ -2797,6 +2827,11 @@
           <t>반도체/IT, 자동차부품 | 투자기업: 테스나, 브이디에스, 에임시스템</t>
         </is>
       </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>https://www.acelp.co.kr:443/superboard/data/siteconfig/2021041419394616183967867220.png</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="14.25" customHeight="1">
       <c r="A51" s="6" t="n">
@@ -2893,6 +2928,11 @@
           <t>미디어/콘텐츠, 전자상거래, 엔터테인먼트 | 투자기업: 리디북스, 번개장터</t>
         </is>
       </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>https://www.praxiscp.com/img/og_logo.gif</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="14.25" customHeight="1">
       <c r="A53" s="6" t="n">
@@ -2941,6 +2981,11 @@
           <t>북미중견기업대출, 부동산담보대출, M&amp;A</t>
         </is>
       </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>http://www.amberstoneam.com/theme/responsive_amberstoneam/include/img/thumnail.png</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="14.25" customHeight="1">
       <c r="A54" s="6" t="n">
@@ -3373,6 +3418,11 @@
           <t>조선해양, 운수, 의료, 기술용역 | 투자기업: 현대힘스, 금남고속, 중부고속, 케어랩스, 크레템</t>
         </is>
       </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>http://jnpef.com/images/sns_link.png</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
       <c r="A63" s="6" t="n">
@@ -3858,6 +3908,11 @@
           <t>바이오테크, 자동차부품, 엔지니어링 | 투자기업: 마이크로바이오틱스, 한양소재</t>
         </is>
       </c>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t>https://www.paratusinvestment.com/img/common/img.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="6" t="n">
@@ -4530,6 +4585,11 @@
           <t>제약 | 투자기업: 한미사이언스</t>
         </is>
       </c>
+      <c r="O86" t="inlineStr">
+        <is>
+          <t>https://www.ldpartners.co.kr/images/common/meta_img.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="87" ht="14.25" customHeight="1">
       <c r="A87" s="6" t="n">
@@ -4723,6 +4783,11 @@
           <t>전기자동차배터리, 에너지저장시스템 | 투자기업: SK On, Key Capture Energy</t>
         </is>
       </c>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>https://stellainv.com/wp-content/uploads/2025/11/Frame-427322446.png</t>
+        </is>
+      </c>
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="6" t="n">
@@ -4963,6 +5028,11 @@
           <t>기술, 헬스케어, 소비재, 금융, 에너지</t>
         </is>
       </c>
+      <c r="O95" t="inlineStr">
+        <is>
+          <t>http://static1.squarespace.com/static/61385885427d7a43ba5e7a89/t/613859d5fc9a13700023e5f9/1770946419285/DSPE+logo.png?format=1500w</t>
+        </is>
+      </c>
     </row>
     <row r="96" ht="14.25" customHeight="1">
       <c r="A96" s="6" t="n">
@@ -5156,6 +5226,11 @@
           <t>바이오, 의료기기, 전자/반도체 | 투자기업: 에이프로젠, 씨벤티지, 코렌, 성호전자</t>
         </is>
       </c>
+      <c r="O99" t="inlineStr">
+        <is>
+          <t>http://www.laic.kr/img/logo_default.gif</t>
+        </is>
+      </c>
     </row>
     <row r="100" ht="14.25" customHeight="1">
       <c r="A100" s="6" t="n">
@@ -5672,6 +5747,11 @@
         <v>1</v>
       </c>
       <c r="N110" s="11" t="n"/>
+      <c r="O110" t="inlineStr">
+        <is>
+          <t>http://www.skscredit.com/bc.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="111" ht="14.25" customHeight="1">
       <c r="A111" s="6" t="n">
@@ -5813,6 +5893,11 @@
           <t>스타트업, B2B, HR Tech, 라이프스타일 | 투자기업: 리멤버, 카시나, 팀스파르타, 숨고</t>
         </is>
       </c>
+      <c r="O113" t="inlineStr">
+        <is>
+          <t>https://www.arknpartners.com/static/images/thumbnail.png</t>
+        </is>
+      </c>
     </row>
     <row r="114" ht="25.5" customHeight="1">
       <c r="A114" s="6" t="n">
@@ -6001,6 +6086,11 @@
           <t>헬스케어, 진단, AI/분석 | 투자기업: 그린벳, 이니바이오</t>
         </is>
       </c>
+      <c r="O117" t="inlineStr">
+        <is>
+          <t>http://www.synaptic-investment.com/images/common/meta_img.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="118" ht="14.25" customHeight="1">
       <c r="A118" s="6" t="n">
@@ -6550,6 +6640,11 @@
           <t>전자상거래, 의료 | 투자기업: 큐텐(Qoo10), 진이어스</t>
         </is>
       </c>
+      <c r="O129" t="inlineStr">
+        <is>
+          <t>https://metistone.com/file/1426167083</t>
+        </is>
+      </c>
     </row>
     <row r="130" ht="14.25" customHeight="1">
       <c r="A130" s="6" t="n">
@@ -6730,6 +6825,11 @@
         <v>0</v>
       </c>
       <c r="N133" s="11" t="n"/>
+      <c r="O133" t="inlineStr">
+        <is>
+          <t>https://assets.softr-files.com/assets/images/random/og_default_image.png</t>
+        </is>
+      </c>
     </row>
     <row r="134" ht="14.25" customHeight="1">
       <c r="A134" s="6" t="n">
@@ -8182,6 +8282,11 @@
         <v>0</v>
       </c>
       <c r="N164" s="11" t="n"/>
+      <c r="O164" t="inlineStr">
+        <is>
+          <t>https://www.atupartners.com/images/common/logo.png</t>
+        </is>
+      </c>
     </row>
     <row r="165" ht="14.25" customHeight="1">
       <c r="A165" s="6" t="n">
@@ -8278,6 +8383,11 @@
           <t>항공, 소비재, 산업, 환경/에너지 | 투자기업: 에어프레미아</t>
         </is>
       </c>
+      <c r="O166" t="inlineStr">
+        <is>
+          <t>http://www.pavilioninv.com/bc.png</t>
+        </is>
+      </c>
     </row>
     <row r="167" ht="14.25" customHeight="1">
       <c r="A167" s="6" t="n">
@@ -8910,6 +9020,11 @@
         <v>0</v>
       </c>
       <c r="N180" s="11" t="n"/>
+      <c r="O180" t="inlineStr">
+        <is>
+          <t>https://lh3.googleusercontent.com/sitesv/APaQ0SSJ-EYEHOliDwveFWjJ2Y5_67uVKCeA91wCdITpV4A5uaT2nP8daJCcHqEUjYQNlphcXcV72NiDA5Hn28uw0why4Wboj6i5xxeDX0NCFk3XnRqED5kiVP5eXeORbPBcM2804Br9EADtOXXEZQxGSbTpF_yr86znNVFb7UVjJTfy2ONP-Wz2WYx6x-WOAUXSlcTX3w=w1280</t>
+        </is>
+      </c>
     </row>
     <row r="181" ht="14.25" customHeight="1">
       <c r="A181" s="6" t="n">
@@ -8998,6 +9113,11 @@
         <v>0</v>
       </c>
       <c r="N182" s="11" t="n"/>
+      <c r="O182" t="inlineStr">
+        <is>
+          <t>https://tychepartners.co.kr/opengraph.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="183" ht="14.25" customHeight="1">
       <c r="A183" s="6" t="n">
@@ -9494,6 +9614,11 @@
           <t>콜드체인물류, 명품이커머스, 위성영상, AI반도체 | 투자기업: 에스랩아시아, 발란, 콘텍, 오픈엣지</t>
         </is>
       </c>
+      <c r="O193" t="inlineStr">
+        <is>
+          <t>https://cdn.imweb.me/upload/S202105189780c6de5e170/8b771026799d4.png</t>
+        </is>
+      </c>
     </row>
     <row r="194" ht="14.25" customHeight="1">
       <c r="A194" s="6" t="n">
@@ -9582,6 +9707,11 @@
         <v>0</v>
       </c>
       <c r="N195" s="11" t="n"/>
+      <c r="O195" t="inlineStr">
+        <is>
+          <t>https://www.wwg.kr/images/2024/10/GWhr5d1DdKZU6719ca0d7377f2.84256249.png</t>
+        </is>
+      </c>
     </row>
     <row r="196" ht="14.25" customHeight="1">
       <c r="A196" s="6" t="n">
@@ -9626,6 +9756,11 @@
         <v>2</v>
       </c>
       <c r="N196" s="11" t="n"/>
+      <c r="O196" t="inlineStr">
+        <is>
+          <t>http://www.avespartners.com/img/aves_logo_big.png</t>
+        </is>
+      </c>
     </row>
     <row r="197" ht="14.25" customHeight="1">
       <c r="A197" s="6" t="n">
@@ -9758,6 +9893,11 @@
         <v>0</v>
       </c>
       <c r="N199" s="11" t="n"/>
+      <c r="O199" t="inlineStr">
+        <is>
+          <t>https://pscp.co.kr/wp-content/uploads/2024/09/pscp-logo.png</t>
+        </is>
+      </c>
     </row>
     <row r="200" ht="14.25" customHeight="1">
       <c r="A200" s="6" t="n">
@@ -9890,6 +10030,11 @@
         <v>0</v>
       </c>
       <c r="N202" s="11" t="n"/>
+      <c r="O202" t="inlineStr">
+        <is>
+          <t>http://www.bankerstreet.com/sh_img/hd/top_menu/logo.png</t>
+        </is>
+      </c>
     </row>
     <row r="203" ht="14.25" customHeight="1">
       <c r="A203" s="6" t="n">
@@ -10466,6 +10611,11 @@
         <v>0</v>
       </c>
       <c r="N215" s="11" t="n"/>
+      <c r="O215" t="inlineStr">
+        <is>
+          <t>https://cdn.imweb.me/upload/S20200813df95ba9e20d5e/9e35d1729fe71.png</t>
+        </is>
+      </c>
     </row>
     <row r="216" ht="14.25" customHeight="1">
       <c r="A216" s="6" t="n">
@@ -11082,6 +11232,11 @@
         <v>0</v>
       </c>
       <c r="N229" s="11" t="n"/>
+      <c r="O229" t="inlineStr">
+        <is>
+          <t>http://jcurveinvest.com/logo.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="230" ht="14.25" customHeight="1">
       <c r="A230" s="6" t="n">
@@ -11126,6 +11281,11 @@
         <v>0</v>
       </c>
       <c r="N230" s="11" t="n"/>
+      <c r="O230" t="inlineStr">
+        <is>
+          <t>http://lkpartners.co.kr/theme/business/extend/sections/header/lkti7010_header/img/logo.png?ver=250115</t>
+        </is>
+      </c>
     </row>
     <row r="231" ht="14.25" customHeight="1">
       <c r="A231" s="6" t="n">
@@ -11478,6 +11638,11 @@
         <v>0</v>
       </c>
       <c r="N238" s="11" t="n"/>
+      <c r="O238" t="inlineStr">
+        <is>
+          <t>http://www.mintventures.bio/data/upload/1712292236_OG.png</t>
+        </is>
+      </c>
     </row>
     <row r="239" ht="14.25" customHeight="1">
       <c r="A239" s="6" t="n">
@@ -11962,6 +12127,11 @@
         <v>0</v>
       </c>
       <c r="N249" s="11" t="n"/>
+      <c r="O249" t="inlineStr">
+        <is>
+          <t>https://www.simonefg.co.kr/theme/basic/img/ci.png</t>
+        </is>
+      </c>
     </row>
     <row r="250" ht="14.25" customHeight="1">
       <c r="A250" s="6" t="n">
@@ -12754,6 +12924,11 @@
         <v>0</v>
       </c>
       <c r="N267" s="11" t="n"/>
+      <c r="O267" t="inlineStr">
+        <is>
+          <t>http://oraclevc.co.kr/assets/img/001.png</t>
+        </is>
+      </c>
     </row>
     <row r="268" ht="14.25" customHeight="1">
       <c r="A268" s="6" t="n">
@@ -12895,6 +13070,11 @@
         <v>0</v>
       </c>
       <c r="N270" s="11" t="n"/>
+      <c r="O270" t="inlineStr">
+        <is>
+          <t>https://cdn.imweb.me/upload/S201904295cc6b4b6c8d89/8ca3f906f65e4.png</t>
+        </is>
+      </c>
     </row>
     <row r="271" ht="14.25" customHeight="1">
       <c r="A271" s="6" t="n">
@@ -13603,6 +13783,11 @@
         <v>0</v>
       </c>
       <c r="N286" s="11" t="n"/>
+      <c r="O286" t="inlineStr">
+        <is>
+          <t>https://cdn.imweb.me/upload/S20220720d03f1eb427cf9/4da7d4a64c447.png</t>
+        </is>
+      </c>
     </row>
     <row r="287" ht="14.25" customHeight="1">
       <c r="A287" s="6" t="n">
@@ -13911,6 +14096,11 @@
         <v>0</v>
       </c>
       <c r="N293" s="11" t="n"/>
+      <c r="O293" t="inlineStr">
+        <is>
+          <t>https://www.investwells.com/img/logo-b.svg</t>
+        </is>
+      </c>
     </row>
     <row r="294" ht="14.25" customHeight="1">
       <c r="A294" s="6" t="n">
@@ -14087,6 +14277,11 @@
         <v>0</v>
       </c>
       <c r="N297" s="11" t="n"/>
+      <c r="O297" t="inlineStr">
+        <is>
+          <t>http://harborbricks.co.kr/img/common/logo.png</t>
+        </is>
+      </c>
     </row>
     <row r="298" ht="14.25" customHeight="1">
       <c r="A298" s="6" t="n">
@@ -14351,6 +14546,11 @@
         <v>0</v>
       </c>
       <c r="N303" s="11" t="n"/>
+      <c r="O303" t="inlineStr">
+        <is>
+          <t>https://www.koreitasset.com/assets/global/images/SEO_img_1200X630_02.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="304" ht="14.25" customHeight="1">
       <c r="A304" s="6" t="n">
@@ -14571,6 +14771,11 @@
         <v>0</v>
       </c>
       <c r="N308" s="11" t="n"/>
+      <c r="O308" t="inlineStr">
+        <is>
+          <t>https://gorillape.com/img/meta_image.png</t>
+        </is>
+      </c>
     </row>
     <row r="309" ht="14.25" customHeight="1">
       <c r="A309" s="6" t="n">
@@ -14615,6 +14820,11 @@
         <v>0</v>
       </c>
       <c r="N309" s="11" t="n"/>
+      <c r="O309" t="inlineStr">
+        <is>
+          <t>http://www.theturningpoint.co.kr/upload/site/20240603041427_1f09178b.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="310" ht="14.25" customHeight="1">
       <c r="A310" s="6" t="n">
@@ -15143,6 +15353,11 @@
         <v>1</v>
       </c>
       <c r="N321" s="11" t="n"/>
+      <c r="O321" t="inlineStr">
+        <is>
+          <t>http://www.m-vc.co.kr/uploads/meta/63087fa3afd30.png</t>
+        </is>
+      </c>
     </row>
     <row r="322" ht="14.25" customHeight="1">
       <c r="A322" s="6" t="n">
@@ -15187,6 +15402,11 @@
         <v>0</v>
       </c>
       <c r="N322" s="11" t="n"/>
+      <c r="O322" t="inlineStr">
+        <is>
+          <t>https://partners.wadiz.kr/opengraph-image.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="323" ht="14.25" customHeight="1">
       <c r="A323" s="6" t="n">
@@ -15275,6 +15495,11 @@
         <v>2</v>
       </c>
       <c r="N324" s="11" t="n"/>
+      <c r="O324" t="inlineStr">
+        <is>
+          <t>http://daylipartners.website.ne.kr/images/sns_link.png</t>
+        </is>
+      </c>
     </row>
     <row r="325" ht="14.25" customHeight="1">
       <c r="A325" s="6" t="n">
@@ -15407,6 +15632,11 @@
         <v>0</v>
       </c>
       <c r="N327" s="11" t="n"/>
+      <c r="O327" t="inlineStr">
+        <is>
+          <t>https://tychepe.com/wp-content/uploads/2022/04/티케인베스트먼트-로고1.png</t>
+        </is>
+      </c>
     </row>
     <row r="328" ht="14.25" customHeight="1">
       <c r="A328" s="6" t="n">
@@ -15847,6 +16077,11 @@
         <v>1</v>
       </c>
       <c r="N337" s="11" t="n"/>
+      <c r="O337" t="inlineStr">
+        <is>
+          <t>http://invictusasia.com/images/kakao.png</t>
+        </is>
+      </c>
     </row>
     <row r="338" ht="14.25" customHeight="1">
       <c r="A338" s="6" t="n">
@@ -15891,6 +16126,11 @@
         <v>0</v>
       </c>
       <c r="N338" s="11" t="n"/>
+      <c r="O338" t="inlineStr">
+        <is>
+          <t>http://www.openwaterinv.co.kr/off/img/27.png</t>
+        </is>
+      </c>
     </row>
     <row r="339" ht="14.25" customHeight="1">
       <c r="A339" s="6" t="n">
@@ -15935,6 +16175,11 @@
         <v>0</v>
       </c>
       <c r="N339" s="11" t="n"/>
+      <c r="O339" t="inlineStr">
+        <is>
+          <t>https://launchpack-storage.s3.ap-northeast-2.amazonaws.com/media/ccvc/non-path/42746849.png</t>
+        </is>
+      </c>
     </row>
     <row r="340" ht="14.25" customHeight="1">
       <c r="A340" s="6" t="n">

</xml_diff>